<commit_message>
More CSS work, edited pages to have matching headers
Also added name attributes to all inputs on addCourse. Working on getting familiar with CSS and having all pages aligned. Note: I removed the <main> tags from the addinstructor and enrollstudent pages. They were causing the CSS to not be applied, and since these pages only have the form in them (for now), we don't have any additional content in these pages... so I'm not sure we need the main tags, but we can talk to Dr. Williamson about it soon to make sure
</commit_message>
<xml_diff>
--- a/CSCI330 Group Project Task Tracker.xlsx
+++ b/CSCI330 Group Project Task Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30502"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://marietta0-my.sharepoint.com/personal/mca003_marietta_edu/Documents/Junior Year/F26/CSCI330/Group Project/Web-Design-and-Programming-GroupWork/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C5AEFBD-5EE4-4783-87B6-0456A0AA740F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{2C5AEFBD-5EE4-4783-87B6-0456A0AA740F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C92F1EB6-8CC2-46E5-8CDC-1ACBC169B15B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="24">
   <si>
     <t>Task</t>
   </si>
@@ -99,13 +99,25 @@
   </si>
   <si>
     <t>Group Peer Evaluations</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Last Updated</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>HTML done, needs CSS applied</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,11 +154,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -481,15 +494,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4840B388-0DE6-4C53-AF10-25A76A976816}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.6">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -499,8 +514,14 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -508,10 +529,17 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2">
+        <f>DATE(2026,9,17)</f>
+        <v>46282</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -522,7 +550,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -533,7 +561,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -541,10 +569,17 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2">
+        <f>DATE(2026,9,17)</f>
+        <v>46282</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -555,7 +590,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -566,7 +601,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -574,10 +609,14 @@
         <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+        <v>5</v>
+      </c>
+      <c r="D8" s="2">
+        <f>DATE(2026,9,17)</f>
+        <v>46282</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -588,7 +627,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -599,7 +638,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -610,7 +649,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
Remove old copy of tracker
</commit_message>
<xml_diff>
--- a/CSCI330 Group Project Task Tracker.xlsx
+++ b/CSCI330 Group Project Task Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30520"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://marietta0-my.sharepoint.com/personal/mca003_marietta_edu/Documents/Junior Year/F26/CSCI330/Group Project/Web-Design-and-Programming-GroupWork/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="8_{2C5AEFBD-5EE4-4783-87B6-0456A0AA740F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4F3F39E-77E7-4E3D-9235-29C9185504D7}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F6A5FAB-AFE7-47E1-ACB1-A9D1F95A9BF3}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="41">
   <si>
     <t>Task</t>
   </si>
@@ -50,80 +50,125 @@
     <t>Progress</t>
   </si>
   <si>
+    <t>Home page</t>
+  </si>
+  <si>
+    <t>Maisee</t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>Enroll student</t>
+  </si>
+  <si>
+    <t>Beatrice</t>
+  </si>
+  <si>
+    <t>Add instructor</t>
+  </si>
+  <si>
+    <t>Add course</t>
+  </si>
+  <si>
+    <t>Not started</t>
+  </si>
+  <si>
+    <t>Register course</t>
+  </si>
+  <si>
+    <t>Drew</t>
+  </si>
+  <si>
+    <t>Drop course</t>
+  </si>
+  <si>
+    <t>CSS</t>
+  </si>
+  <si>
+    <t>Manuals</t>
+  </si>
+  <si>
+    <t>README file</t>
+  </si>
+  <si>
+    <t>AI Usage Report</t>
+  </si>
+  <si>
+    <t>ALL</t>
+  </si>
+  <si>
+    <t>Group Peer Evaluations</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
     <t>Last Updated</t>
   </si>
   <si>
     <t>Notes</t>
   </si>
   <si>
-    <t>Home page</t>
-  </si>
-  <si>
-    <t>Maisee</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
     <t>HTML done, needs CSS applied</t>
   </si>
   <si>
-    <t>Enroll student</t>
-  </si>
-  <si>
-    <t>Beatrice</t>
-  </si>
-  <si>
-    <t>Need to apply CSS</t>
-  </si>
-  <si>
-    <t>Add instructor</t>
-  </si>
-  <si>
-    <t>Add course</t>
-  </si>
-  <si>
-    <t>Register course</t>
-  </si>
-  <si>
-    <t>Drew</t>
-  </si>
-  <si>
-    <t>Drop course</t>
-  </si>
-  <si>
-    <t>CSS</t>
-  </si>
-  <si>
-    <t>In progress</t>
-  </si>
-  <si>
-    <t>Manuals</t>
-  </si>
-  <si>
-    <t>Done with user manual(needs css),started programmer manual</t>
-  </si>
-  <si>
-    <t>README file</t>
-  </si>
-  <si>
-    <t>AI Usage Report</t>
-  </si>
-  <si>
-    <t>ALL</t>
-  </si>
-  <si>
-    <t>Group Peer Evaluations</t>
-  </si>
-  <si>
-    <t>Not started</t>
+    <t>need to apply css</t>
+  </si>
+  <si>
+    <t>Maisee, Beatrice</t>
+  </si>
+  <si>
+    <t>MODULE TWO</t>
+  </si>
+  <si>
+    <t>Enroll Student form display</t>
+  </si>
+  <si>
+    <t>Add Instructor form display</t>
+  </si>
+  <si>
+    <t>Add Course form display</t>
+  </si>
+  <si>
+    <t>Register Course form display</t>
+  </si>
+  <si>
+    <t>Drop Course form display</t>
+  </si>
+  <si>
+    <t>Updating manuals</t>
+  </si>
+  <si>
+    <t>Update select list display for Add Course</t>
+  </si>
+  <si>
+    <t>Enroll Student validation (4 rules)</t>
+  </si>
+  <si>
+    <t>Add Instructor validation (4 rules)</t>
+  </si>
+  <si>
+    <t>Add Course validation (9 rules)</t>
+  </si>
+  <si>
+    <t>Register Course validation (6 rules)</t>
+  </si>
+  <si>
+    <t>Drop Course validation (6 rules)</t>
+  </si>
+  <si>
+    <t>Beatrice &amp; Maisee</t>
+  </si>
+  <si>
+    <t>Any updates/fixes from Module 1 grade</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -139,6 +184,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -148,7 +201,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -156,16 +209,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -500,17 +574,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4840B388-0DE6-4C53-AF10-25A76A976816}">
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:E29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="53.85546875" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -521,182 +595,361 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D2" s="2">
         <f>DATE(2026,9,17)</f>
         <v>46282</v>
       </c>
       <c r="E2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2">
+        <v>46284</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2">
+        <v>46285</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="2">
-        <v>46283</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="2">
-        <v>46283</v>
-      </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D5" s="2">
         <f>DATE(2026,9,17)</f>
         <v>46282</v>
       </c>
       <c r="E5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2">
+        <v>46285</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2">
+        <v>46285</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="2">
-        <v>46284</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="2">
-        <v>46284</v>
-      </c>
-      <c r="E7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>17</v>
-      </c>
       <c r="B8" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D8" s="2">
         <f>DATE(2026,9,17)</f>
         <v>46282</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="2">
+        <v>46284</v>
+      </c>
+      <c r="E9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>19</v>
       </c>
-      <c r="B9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="B12" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="2">
-        <v>46283</v>
-      </c>
-      <c r="E9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" t="s">
-        <v>25</v>
+      <c r="C27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A13:E13"/>
+  </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C12" xr:uid="{1AE900CF-695F-49FE-919B-A3667E9EEDD6}">
       <formula1>"Not started, In progress, Completed, Stuck/need help"</formula1>

</xml_diff>

<commit_message>
Created JavaScript page, added script links to every page, adjusted file organization
Please use the validation.js file to add your validation rules. I also created an AI Usage Report for this module and added it to the folder
</commit_message>
<xml_diff>
--- a/CSCI330 Group Project Task Tracker.xlsx
+++ b/CSCI330 Group Project Task Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://marietta0-my.sharepoint.com/personal/mca003_marietta_edu/Documents/Junior Year/F26/CSCI330/Group Project/Web-Design-and-Programming-GroupWork/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F6A5FAB-AFE7-47E1-ACB1-A9D1F95A9BF3}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11F97A06-0197-42D1-8C01-F10BFDF9B92B}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -193,12 +193,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -228,18 +234,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -762,13 +769,13 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -793,13 +800,13 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="A16" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -848,13 +855,13 @@
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="A21" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -881,13 +888,13 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="A24" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -903,13 +910,13 @@
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="A26" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="5" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Finished addcourse validation, work on pop-up display
I have some questions I need to ask dr. Williamson about for the print display that happens after validation, but it works for now. I will spend time in the next few days working on the course dropdown and then I will wait until next week (once we have more progress) to do the README file.
</commit_message>
<xml_diff>
--- a/CSCI330 Group Project Task Tracker.xlsx
+++ b/CSCI330 Group Project Task Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://marietta0-my.sharepoint.com/personal/mca003_marietta_edu/Documents/Junior Year/F26/CSCI330/Group Project/Web-Design-and-Programming-GroupWork/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11F97A06-0197-42D1-8C01-F10BFDF9B92B}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10CDE41F-018B-4ECA-9E19-1BF481F85B6F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
   </bookViews>
@@ -240,13 +240,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -769,13 +769,13 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -800,14 +800,17 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>10</v>
+      <c r="C16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="2">
+        <v>46315</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -855,13 +858,13 @@
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="3" t="s">
         <v>10</v>
       </c>
     </row>
@@ -888,13 +891,13 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="3" t="s">
         <v>10</v>
       </c>
     </row>
@@ -910,13 +913,13 @@
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="3" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update CSCI330 Group Project Task Tracker.xlsx
</commit_message>
<xml_diff>
--- a/CSCI330 Group Project Task Tracker.xlsx
+++ b/CSCI330 Group Project Task Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://marietta0-my.sharepoint.com/personal/mca003_marietta_edu/Documents/Junior Year/F26/CSCI330/Group Project/Web-Design-and-Programming-GroupWork/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10CDE41F-018B-4ECA-9E19-1BF481F85B6F}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6276C51-32F2-4E3E-B127-9AE165704197}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="42">
   <si>
     <t>Task</t>
   </si>
@@ -162,6 +162,9 @@
   </si>
   <si>
     <t>Any updates/fixes from Module 1 grade</t>
+  </si>
+  <si>
+    <t>Need to ask Williamson about display</t>
   </si>
 </sst>
 </file>
@@ -588,7 +591,7 @@
     <col min="2" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="17.6640625" customWidth="1"/>
     <col min="4" max="4" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
@@ -813,7 +816,7 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>37</v>
       </c>
@@ -824,7 +827,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -835,7 +838,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -846,7 +849,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -857,7 +860,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>29</v>
       </c>
@@ -865,10 +868,16 @@
         <v>4</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+      <c r="D21" s="2">
+        <v>46315</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>30</v>
       </c>
@@ -879,7 +888,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>31</v>
       </c>
@@ -890,7 +899,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>33</v>
       </c>
@@ -901,7 +910,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -912,7 +921,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>16</v>
       </c>
@@ -923,7 +932,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>17</v>
       </c>
@@ -934,7 +943,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>19</v>
       </c>
@@ -945,7 +954,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>40</v>
       </c>

</xml_diff>

<commit_message>
Worked on display lists for day/time
Going to work on a few stylistic issues here, but this works for now. I'm thinking next week we can try to implement some additional validation rules for extra credit (we would need 5 total). I am going to try and get the README file done before Tuesday and then spend time proofreading the manuals and adding in validation rules as mentioned above.
</commit_message>
<xml_diff>
--- a/CSCI330 Group Project Task Tracker.xlsx
+++ b/CSCI330 Group Project Task Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://marietta0-my.sharepoint.com/personal/mca003_marietta_edu/Documents/Junior Year/F26/CSCI330/Group Project/Web-Design-and-Programming-GroupWork/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6276C51-32F2-4E3E-B127-9AE165704197}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3620E8E-5C05-4B15-ADDE-3618234CE928}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="41">
   <si>
     <t>Task</t>
   </si>
@@ -162,9 +162,6 @@
   </si>
   <si>
     <t>Any updates/fixes from Module 1 grade</t>
-  </si>
-  <si>
-    <t>Need to ask Williamson about display</t>
   </si>
 </sst>
 </file>
@@ -196,7 +193,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -206,6 +203,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -237,7 +246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -250,6 +259,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -781,24 +793,24 @@
       <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="A14" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="A15" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="6" t="s">
         <v>10</v>
       </c>
     </row>
@@ -817,46 +829,46 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="A17" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="A18" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="A19" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="A20" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="6" t="s">
         <v>10</v>
       </c>
     </row>
@@ -873,29 +885,27 @@
       <c r="D21" s="2">
         <v>46315</v>
       </c>
-      <c r="E21" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="E21" s="8"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="A22" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="A23" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="7" t="s">
         <v>10</v>
       </c>
     </row>
@@ -911,13 +921,13 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="A25" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="6" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed register course & drop course error messages
</commit_message>
<xml_diff>
--- a/CSCI330 Group Project Task Tracker.xlsx
+++ b/CSCI330 Group Project Task Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30619"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://marietta0-my.sharepoint.com/personal/mca003_marietta_edu/Documents/Junior Year/F26/CSCI330/Group Project/Web-Design-and-Programming-GroupWork/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="133" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7EC3BA0-BE38-4A4E-912A-7B6CD69751F7}"/>
+  <xr:revisionPtr revIDLastSave="150" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{410288C3-DFF8-43D2-ABC0-8A2A44450946}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
   </bookViews>
@@ -50,112 +50,112 @@
     <t>Progress</t>
   </si>
   <si>
+    <t>Last Updated</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
     <t>Home page</t>
   </si>
   <si>
     <t>Maisee</t>
   </si>
   <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>HTML done, needs CSS applied</t>
+  </si>
+  <si>
+    <t>Enroll student</t>
+  </si>
+  <si>
+    <t>Beatrice</t>
+  </si>
+  <si>
+    <t>need to apply css</t>
+  </si>
+  <si>
+    <t>Add instructor</t>
+  </si>
+  <si>
+    <t>Add course</t>
+  </si>
+  <si>
+    <t>Register course</t>
+  </si>
+  <si>
+    <t>Drew</t>
+  </si>
+  <si>
+    <t>Drop course</t>
+  </si>
+  <si>
+    <t>CSS</t>
+  </si>
+  <si>
+    <t>Maisee, Beatrice</t>
+  </si>
+  <si>
+    <t>Manuals</t>
+  </si>
+  <si>
+    <t>README file</t>
+  </si>
+  <si>
+    <t>AI Usage Report</t>
+  </si>
+  <si>
+    <t>ALL</t>
+  </si>
+  <si>
+    <t>Group Peer Evaluations</t>
+  </si>
+  <si>
+    <t>MODULE TWO</t>
+  </si>
+  <si>
+    <t>Enroll Student validation (4 rules)</t>
+  </si>
+  <si>
+    <t>Add Instructor validation (4 rules)</t>
+  </si>
+  <si>
+    <t>Add Course validation (9 rules)</t>
+  </si>
+  <si>
+    <t>Register Course validation (6 rules)</t>
+  </si>
+  <si>
     <t>In progress</t>
   </si>
   <si>
-    <t>Enroll student</t>
-  </si>
-  <si>
-    <t>Beatrice</t>
-  </si>
-  <si>
-    <t>Add instructor</t>
-  </si>
-  <si>
-    <t>Add course</t>
+    <t>Drop Course validation (6 rules)</t>
+  </si>
+  <si>
+    <t>Enroll Student form display</t>
+  </si>
+  <si>
+    <t>Add Instructor form display</t>
+  </si>
+  <si>
+    <t>Add Course form display</t>
+  </si>
+  <si>
+    <t>Register Course form display</t>
   </si>
   <si>
     <t>Not started</t>
   </si>
   <si>
-    <t>Register course</t>
-  </si>
-  <si>
-    <t>Drew</t>
-  </si>
-  <si>
-    <t>Drop course</t>
-  </si>
-  <si>
-    <t>CSS</t>
-  </si>
-  <si>
-    <t>Manuals</t>
-  </si>
-  <si>
-    <t>README file</t>
-  </si>
-  <si>
-    <t>AI Usage Report</t>
-  </si>
-  <si>
-    <t>ALL</t>
-  </si>
-  <si>
-    <t>Group Peer Evaluations</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>Last Updated</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>HTML done, needs CSS applied</t>
-  </si>
-  <si>
-    <t>need to apply css</t>
-  </si>
-  <si>
-    <t>Maisee, Beatrice</t>
-  </si>
-  <si>
-    <t>MODULE TWO</t>
-  </si>
-  <si>
-    <t>Enroll Student form display</t>
-  </si>
-  <si>
-    <t>Add Instructor form display</t>
-  </si>
-  <si>
-    <t>Add Course form display</t>
-  </si>
-  <si>
-    <t>Register Course form display</t>
-  </si>
-  <si>
     <t>Drop Course form display</t>
   </si>
   <si>
+    <t>Update select list display for Add Course</t>
+  </si>
+  <si>
     <t>Updating manuals</t>
-  </si>
-  <si>
-    <t>Update select list display for Add Course</t>
-  </si>
-  <si>
-    <t>Enroll Student validation (4 rules)</t>
-  </si>
-  <si>
-    <t>Add Instructor validation (4 rules)</t>
-  </si>
-  <si>
-    <t>Add Course validation (9 rules)</t>
-  </si>
-  <si>
-    <t>Register Course validation (6 rules)</t>
-  </si>
-  <si>
-    <t>Drop Course validation (6 rules)</t>
   </si>
   <si>
     <t>Beatrice &amp; Maisee</t>
@@ -168,7 +168,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -608,16 +608,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4840B388-0DE6-4C53-AF10-25A76A976816}">
   <dimension ref="A1:E29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="34.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" customWidth="1"/>
-    <col min="4" max="4" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15.6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -628,391 +628,391 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D2" s="2">
         <f>DATE(2026,9,17)</f>
         <v>46282</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D3" s="2">
         <v>46284</v>
       </c>
       <c r="E3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D4" s="2">
         <v>46285</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D5" s="2">
         <f>DATE(2026,9,17)</f>
         <v>46282</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D6" s="2">
         <v>46285</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D7" s="2">
         <v>46285</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D8" s="2">
         <f>DATE(2026,9,17)</f>
         <v>46282</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D9" s="2">
         <v>46284</v>
       </c>
       <c r="E9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="11" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
-        <v>26</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
       <c r="E13" s="11"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5">
       <c r="A14" s="9" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="8" t="s">
         <v>10</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>7</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5">
       <c r="A15" s="9" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="8" t="s">
         <v>10</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>7</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5">
       <c r="A16" s="4" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D16" s="5">
         <v>46315</v>
       </c>
       <c r="E16" s="3"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5">
       <c r="A17" s="6" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>10</v>
+        <v>15</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5">
       <c r="A18" s="6" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>10</v>
+        <v>15</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5">
       <c r="A19" s="9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" s="8" t="s">
         <v>10</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>7</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5">
       <c r="A20" s="9" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="8" t="s">
         <v>10</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>7</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5">
       <c r="A21" s="4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D21" s="5">
         <v>46315</v>
       </c>
       <c r="E21" s="3"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5">
       <c r="A22" s="6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5">
       <c r="A23" s="6" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5">
       <c r="A24" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D24" s="5">
         <v>46317</v>
       </c>
       <c r="E24" s="3"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5">
       <c r="A25" s="9" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>39</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5">
       <c r="A26" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5">
       <c r="A27" s="3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5">
       <c r="A28" s="3" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5">
       <c r="A29" s="3" t="s">
         <v>40</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>

</xml_diff>